<commit_message>
add some demo templates
</commit_message>
<xml_diff>
--- a/數據類型映射表.xlsx
+++ b/數據類型映射表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Develop\Workspace\OpenSource\DevHelper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B713F9C-5C9E-450D-BCFB-9C604858D5FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99827C77-367E-4216-9936-82686A2D848B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1103" yWindow="1103" windowWidth="17100" windowHeight="9217" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="48">
   <si>
     <t>C++</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -212,6 +212,10 @@
   </si>
   <si>
     <t>byte[m * maxlen + 1]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>String</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -697,7 +701,7 @@
         <v>46</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>14</v>
@@ -726,7 +730,7 @@
         <v>46</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>15</v>

</xml_diff>